<commit_message>
Dados de entrada valores avaliação 2
</commit_message>
<xml_diff>
--- a/CST/Dados de entrada.xlsx
+++ b/CST/Dados de entrada.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Nós</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t xml:space="preserve">t (espessura)</t>
+  </si>
+  <si>
+    <t>-0.5</t>
   </si>
 </sst>
 </file>
@@ -152,12 +155,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -757,312 +760,408 @@
       <c r="J3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="K3" s="6" t="s">
+      <c r="K3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="L3" s="6" t="s">
+      <c r="L3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="M3" s="4" t="s">
         <v>10</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="O3" s="6" t="s">
+      <c r="O3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="P3" s="6" t="s">
+      <c r="P3" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7">
-        <v>1</v>
-      </c>
-      <c r="B4" s="7">
-        <v>0</v>
-      </c>
-      <c r="C4" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D4" s="7">
-        <v>0</v>
-      </c>
-      <c r="E4" s="7">
-        <v>0</v>
-      </c>
-      <c r="F4" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" s="7">
-        <v>0</v>
-      </c>
-      <c r="J4" s="7">
-        <v>1</v>
-      </c>
-      <c r="K4" s="7">
-        <v>1</v>
-      </c>
-      <c r="L4" s="7">
+      <c r="A4" s="6">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6">
+        <v>0</v>
+      </c>
+      <c r="C4" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6">
+        <v>0</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0</v>
+      </c>
+      <c r="F4" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6">
+        <v>1</v>
+      </c>
+      <c r="K4" s="6">
+        <v>1</v>
+      </c>
+      <c r="L4" s="6">
         <v>2</v>
       </c>
-      <c r="M4" s="7">
+      <c r="M4" s="6">
+        <v>6</v>
+      </c>
+      <c r="N4" s="7">
+        <v>1</v>
+      </c>
+      <c r="O4" s="7">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="P4" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6">
         <v>3</v>
       </c>
-      <c r="N4" s="8">
-        <v>210000</v>
-      </c>
-      <c r="O4" s="8">
+      <c r="C5" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6">
+        <v>0</v>
+      </c>
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5" s="6">
+        <v>0</v>
+      </c>
+      <c r="J5" s="6">
+        <v>2</v>
+      </c>
+      <c r="K5" s="6">
+        <v>1</v>
+      </c>
+      <c r="L5" s="6">
+        <v>6</v>
+      </c>
+      <c r="M5" s="6">
+        <v>5</v>
+      </c>
+      <c r="N5" s="7">
+        <v>1</v>
+      </c>
+      <c r="O5" s="7">
         <v>0.29999999999999999</v>
       </c>
-      <c r="P4" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="7">
+      <c r="P5" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6">
+        <v>6</v>
+      </c>
+      <c r="C6" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>3</v>
+      </c>
+      <c r="K6" s="6">
         <v>2</v>
       </c>
-      <c r="B5" s="7">
-        <v>100</v>
-      </c>
-      <c r="C5" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D5" s="7">
-        <v>5000</v>
-      </c>
-      <c r="E5" s="7">
-        <v>0</v>
-      </c>
-      <c r="F5" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G5" s="7">
-        <v>0</v>
-      </c>
-      <c r="J5" s="7">
+      <c r="L6" s="6">
+        <v>3</v>
+      </c>
+      <c r="M6" s="6">
+        <v>7</v>
+      </c>
+      <c r="N6" s="7">
+        <v>1</v>
+      </c>
+      <c r="O6" s="7">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="P6" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6">
+        <v>4</v>
+      </c>
+      <c r="B7" s="6">
+        <v>9</v>
+      </c>
+      <c r="C7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0</v>
+      </c>
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" s="6">
+        <v>4</v>
+      </c>
+      <c r="K7" s="6">
         <v>2</v>
       </c>
-      <c r="K5" s="7">
-        <v>1</v>
-      </c>
-      <c r="L5" s="7">
+      <c r="L7" s="6">
+        <v>7</v>
+      </c>
+      <c r="M7" s="6">
+        <v>6</v>
+      </c>
+      <c r="N7" s="7">
+        <v>1</v>
+      </c>
+      <c r="O7" s="7">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="P7" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6">
+        <v>0</v>
+      </c>
+      <c r="C8" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0</v>
+      </c>
+      <c r="E8" s="6">
         <v>3</v>
       </c>
-      <c r="M5" s="7">
+      <c r="F8" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <v>5</v>
+      </c>
+      <c r="K8" s="6">
+        <v>3</v>
+      </c>
+      <c r="L8" s="6">
         <v>4</v>
       </c>
-      <c r="N5" s="8">
-        <v>210000</v>
-      </c>
-      <c r="O5" s="8">
+      <c r="M8" s="6">
+        <v>8</v>
+      </c>
+      <c r="N8" s="7">
+        <v>1</v>
+      </c>
+      <c r="O8" s="7">
         <v>0.29999999999999999</v>
       </c>
-      <c r="P5" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="7">
+      <c r="P8" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6">
+        <v>6</v>
+      </c>
+      <c r="B9" s="6">
         <v>3</v>
       </c>
-      <c r="B6" s="7">
-        <v>100</v>
-      </c>
-      <c r="C6" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D6" s="7">
-        <v>5000</v>
-      </c>
-      <c r="E6" s="7">
-        <v>100</v>
-      </c>
-      <c r="F6" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="7">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7"/>
-      <c r="M6" s="7"/>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="7"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="7">
-        <v>4</v>
-      </c>
-      <c r="B7" s="7">
-        <v>0</v>
-      </c>
-      <c r="C7" s="7" t="b">
-        <v>1</v>
-      </c>
-      <c r="D7" s="7">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7">
-        <v>100</v>
-      </c>
-      <c r="F7" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" s="7">
-        <v>0</v>
-      </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="7"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="7"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" s="7"/>
-      <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="7"/>
+      <c r="C9" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0</v>
+      </c>
+      <c r="E9" s="6">
+        <v>3</v>
+      </c>
+      <c r="F9" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <v>6</v>
+      </c>
+      <c r="K9" s="6">
+        <v>3</v>
+      </c>
+      <c r="L9" s="6">
+        <v>8</v>
+      </c>
+      <c r="M9" s="6">
+        <v>7</v>
+      </c>
+      <c r="N9" s="7">
+        <v>1</v>
+      </c>
+      <c r="O9" s="7">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="P9" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="7"/>
-      <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
+      <c r="A10" s="6">
+        <v>7</v>
+      </c>
+      <c r="B10" s="6">
+        <v>6</v>
+      </c>
+      <c r="C10" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0</v>
+      </c>
+      <c r="E10" s="6">
+        <v>3</v>
+      </c>
+      <c r="F10" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0</v>
+      </c>
+      <c r="J10" s="6"/>
+      <c r="K10" s="6"/>
+      <c r="L10" s="6"/>
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+      <c r="O10" s="6"/>
+      <c r="P10" s="6"/>
     </row>
     <row r="11">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="7"/>
-      <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="7"/>
+      <c r="A11" s="6">
+        <v>8</v>
+      </c>
+      <c r="B11" s="6">
+        <v>9</v>
+      </c>
+      <c r="C11" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0</v>
+      </c>
+      <c r="E11" s="6">
+        <v>3</v>
+      </c>
+      <c r="F11" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="6"/>
+      <c r="K11" s="6"/>
+      <c r="L11" s="6"/>
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+      <c r="O11" s="6"/>
+      <c r="P11" s="6"/>
     </row>
     <row r="12">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6"/>
+      <c r="J12" s="6"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="6"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="6"/>
     </row>
     <row r="13">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" s="7"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
-      <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" s="6"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="6"/>
     </row>
     <row r="14">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7"/>
-      <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-      <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="7"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6"/>
+      <c r="J14" s="6"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="6"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1079,7 +1178,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1" disablePrompts="0">
-        <x14:dataValidation xr:uid="{000C00CB-00A8-4AA5-8591-00E000A100A0}" type="list" allowBlank="1" error="Esse nó não foi definido na tabela de nós." errorStyle="stop" errorTitle="Nó não encontrado" imeMode="noControl" operator="between" showDropDown="1" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00200002-0025-409A-A94B-00D000AC003E}" type="list" allowBlank="1" error="Esse nó não foi definido na tabela de nós." errorStyle="stop" errorTitle="Nó não encontrado" imeMode="noControl" operator="between" showDropDown="1" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>$A$4:$A$14</xm:f>
           </x14:formula1>

</xml_diff>